<commit_message>
Absensi 5 September 2026 (3 mark) + Dareen & Axelle keluar sekolah
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi T.P 2026-2027/Absensi September 2026 Saturday 08_33_12.xlsx
+++ b/PC-06/docs/Absensi T.P 2026-2027/Absensi September 2026 Saturday 08_33_12.xlsx
@@ -1135,8 +1135,16 @@
       </c>
       <c r="D10" s="12" t="n"/>
       <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H10" s="12" t="n"/>
       <c r="I10" s="12" t="n"/>
       <c r="J10" s="12" t="n"/>
@@ -4370,8 +4378,16 @@
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
@@ -4462,7 +4478,11 @@
         </is>
       </c>
       <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
@@ -4556,7 +4576,11 @@
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="n"/>
       <c r="J17" s="8" t="n"/>
@@ -4692,7 +4716,11 @@
         </is>
       </c>
       <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F20" s="8" t="n"/>
       <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
@@ -5072,7 +5100,11 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E28" s="8" t="n"/>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
@@ -5394,9 +5426,21 @@
         </is>
       </c>
       <c r="D35" s="8" t="n"/>
-      <c r="E35" s="8" t="n"/>
-      <c r="F35" s="8" t="n"/>
-      <c r="G35" s="8" t="n"/>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H35" s="8" t="n"/>
       <c r="I35" s="8" t="n"/>
       <c r="J35" s="8" t="n"/>
@@ -8240,7 +8284,11 @@
         </is>
       </c>
       <c r="D27" s="8" t="n"/>
-      <c r="E27" s="8" t="n"/>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
@@ -11213,7 +11261,11 @@
         </is>
       </c>
       <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
@@ -11399,7 +11451,11 @@
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="n"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>

</xml_diff>